<commit_message>
Finished basic subsectors, working on DSD
</commit_message>
<xml_diff>
--- a/[deprecated]/Residential/Ontario/Residential appliances.xlsx
+++ b/[deprecated]/Residential/Ontario/Residential appliances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/daniel_posen_utoronto_ca/Documents/Academia/File Sharing/Alliance Mission - TEMOA/Full team - TEMOA/TEMOA model and data/Data sources/Buildings/Residential/Ontario/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/buildings_sector/[deprecated]/Residential/Ontario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:40009_{CB50274A-2E39-44CA-935F-6467133D2C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1096CE5C-D188-49DA-BC62-4305916BF7AE}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:40009_{CB50274A-2E39-44CA-935F-6467133D2C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8DB6639-F324-4CF5-B029-AD0AFA1AF5FC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="4" r:id="rId1"/>
@@ -29,8 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -519,15 +517,15 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="7">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0"/>
-    <numFmt numFmtId="166" formatCode="0.00000"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="#,##0.000"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="169" formatCode="#,##0.000"/>
+    <numFmt numFmtId="170" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -811,7 +809,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="73">
@@ -847,10 +845,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
@@ -860,8 +858,8 @@
     <xf numFmtId="1" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -873,12 +871,12 @@
     <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -890,13 +888,13 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -907,21 +905,21 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1545,14 +1543,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
     <col min="3" max="9" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
@@ -1581,7 +1579,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2020</v>
       </c>
@@ -1613,7 +1611,7 @@
       <c r="J2" s="14"/>
       <c r="K2" s="14"/>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -1651,7 +1649,7 @@
       <c r="J3" s="14"/>
       <c r="K3" s="14"/>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2030</v>
       </c>
@@ -1689,7 +1687,7 @@
       <c r="J4" s="14"/>
       <c r="K4" s="14"/>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2035</v>
       </c>
@@ -1727,7 +1725,7 @@
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2040</v>
       </c>
@@ -1765,7 +1763,7 @@
       <c r="J6" s="14"/>
       <c r="K6" s="14"/>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2045</v>
       </c>
@@ -1803,7 +1801,7 @@
       <c r="J7" s="14"/>
       <c r="K7" s="14"/>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="27">
         <v>2050</v>
       </c>
@@ -1841,7 +1839,7 @@
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="55" t="s">
         <v>9</v>
       </c>
@@ -1868,7 +1866,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1891,7 +1889,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A63EF33D-35AD-4B4A-945F-862DF8CAB4B9}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" customWidth="1"/>
     <col min="2" max="2" width="29.5703125" customWidth="1"/>
@@ -1900,7 +1898,7 @@
     <col min="5" max="5" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1917,7 +1915,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
@@ -1936,7 +1934,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>3</v>
       </c>
@@ -1955,7 +1953,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>4</v>
       </c>
@@ -1974,7 +1972,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>5</v>
       </c>
@@ -1993,7 +1991,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>20</v>
       </c>
@@ -2012,7 +2010,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>22</v>
       </c>
@@ -2031,7 +2029,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>24</v>
       </c>
@@ -2050,7 +2048,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>26</v>
       </c>
@@ -2069,7 +2067,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>28</v>
       </c>
@@ -2091,7 +2089,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>31</v>
       </c>
@@ -2110,7 +2108,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AN58"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.7109375" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" style="50" bestFit="1" customWidth="1"/>
@@ -2139,7 +2137,7 @@
     <col min="37" max="38" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="27" customFormat="1">
+    <row r="1" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
         <v>32</v>
       </c>
@@ -2189,7 +2187,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -2238,7 +2236,7 @@
         <v>4.2620886094699273E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2287,7 +2285,7 @@
         <v>5.2328969490726573E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2336,7 +2334,7 @@
         <v>0.24048268614091131</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -2385,7 +2383,7 @@
         <v>0.441184809132112</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -2434,7 +2432,7 @@
         <v>2.1172849814229233E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -2483,7 +2481,7 @@
         <v>2.3948000888347479E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2532,7 +2530,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="E9" s="69"/>
       <c r="F9" s="69"/>
       <c r="G9" s="69"/>
@@ -2545,7 +2543,7 @@
       <c r="N9" s="68"/>
       <c r="O9" s="68"/>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
         <v>12</v>
       </c>
@@ -2561,7 +2559,7 @@
       <c r="N10" s="68"/>
       <c r="O10" s="68"/>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2602,7 +2600,7 @@
         <v>4.2620886094699273E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>37</v>
       </c>
@@ -2643,7 +2641,7 @@
         <v>4.2620886094699273E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:16">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -2684,7 +2682,7 @@
         <v>5.2328969490726573E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -2725,7 +2723,7 @@
         <v>5.2328969490726573E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -2766,7 +2764,7 @@
         <v>0.24048268614091131</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -2807,7 +2805,7 @@
         <v>0.24048268614091131</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -2848,7 +2846,7 @@
         <v>0.441184809132112</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -2887,7 +2885,7 @@
         <v>0.441184809132112</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -2926,7 +2924,7 @@
         <v>2.1172849814229233E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2965,7 +2963,7 @@
         <v>2.1172849814229233E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:15">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>42</v>
       </c>
@@ -3004,7 +3002,7 @@
         <v>2.1172849814229233E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -3043,7 +3041,7 @@
         <v>2.1172849814229233E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>44</v>
       </c>
@@ -3082,7 +3080,7 @@
         <v>2.1172849814229233E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -3121,7 +3119,7 @@
         <v>2.1172849814229233E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:15">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -3160,7 +3158,7 @@
         <v>2.1172849814229233E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:15">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>46</v>
       </c>
@@ -3199,7 +3197,7 @@
         <v>2.3948000888347479E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:15">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -3238,7 +3236,7 @@
         <v>2.3948000888347479E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:15">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>47</v>
       </c>
@@ -3277,7 +3275,7 @@
         <v>2.3948000888347479E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:15">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>48</v>
       </c>
@@ -3316,7 +3314,7 @@
         <v>2.3948000888347479E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>49</v>
       </c>
@@ -3355,7 +3353,7 @@
         <v>2.3948000888347479E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>27</v>
       </c>
@@ -3394,7 +3392,7 @@
         <v>2.3948000888347479E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:15">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>50</v>
       </c>
@@ -3433,7 +3431,7 @@
         <v>2.3948000888347479E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:40">
+    <row r="33" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>29</v>
       </c>
@@ -3472,10 +3470,10 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="34" spans="1:40">
+    <row r="34" spans="1:40" x14ac:dyDescent="0.25">
       <c r="J34" s="63"/>
     </row>
-    <row r="35" spans="1:40">
+    <row r="35" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A35" s="25" t="s">
         <v>51</v>
       </c>
@@ -3513,7 +3511,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="36" spans="1:40">
+    <row r="36" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>16</v>
       </c>
@@ -3641,7 +3639,7 @@
         <v>R_APP_OTH_APP</v>
       </c>
     </row>
-    <row r="37" spans="1:40">
+    <row r="37" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>37</v>
       </c>
@@ -3757,7 +3755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:40">
+    <row r="38" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>17</v>
       </c>
@@ -3887,7 +3885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:40">
+    <row r="39" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -4002,7 +4000,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:40">
+    <row r="40" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>18</v>
       </c>
@@ -4130,7 +4128,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="41" spans="1:40">
+    <row r="41" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -4243,7 +4241,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="42" spans="1:40">
+    <row r="42" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>19</v>
       </c>
@@ -4373,7 +4371,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="43" spans="1:40">
+    <row r="43" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>40</v>
       </c>
@@ -4488,7 +4486,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="44" spans="1:40">
+    <row r="44" spans="1:40" x14ac:dyDescent="0.25">
       <c r="C44" s="52"/>
       <c r="D44" s="49"/>
       <c r="E44" s="62"/>
@@ -4575,7 +4573,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="45" spans="1:40">
+    <row r="45" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>21</v>
       </c>
@@ -4702,7 +4700,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="46" spans="1:40">
+    <row r="46" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>42</v>
       </c>
@@ -4814,7 +4812,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="47" spans="1:40">
+    <row r="47" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>43</v>
       </c>
@@ -4941,7 +4939,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="48" spans="1:40">
+    <row r="48" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>44</v>
       </c>
@@ -5053,7 +5051,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="49" spans="1:40">
+    <row r="49" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>23</v>
       </c>
@@ -5180,7 +5178,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="50" spans="1:40">
+    <row r="50" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>45</v>
       </c>
@@ -5292,7 +5290,7 @@
         <v>0.18562273222509823</v>
       </c>
     </row>
-    <row r="51" spans="1:40">
+    <row r="51" spans="1:40" x14ac:dyDescent="0.25">
       <c r="D51" s="49"/>
       <c r="E51" s="62"/>
       <c r="F51" s="62"/>
@@ -5327,7 +5325,7 @@
       <c r="AK51" s="24"/>
       <c r="AL51" s="24"/>
     </row>
-    <row r="52" spans="1:40">
+    <row r="52" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>25</v>
       </c>
@@ -5382,7 +5380,7 @@
         <v>2.616364708196383E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:40">
+    <row r="53" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>47</v>
       </c>
@@ -5422,7 +5420,7 @@
         <v>3.3610730508316249E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:40">
+    <row r="54" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>48</v>
       </c>
@@ -5477,7 +5475,7 @@
         <v>1.5841957667984317E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:40">
+    <row r="55" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>49</v>
       </c>
@@ -5517,7 +5515,7 @@
         <v>1.6272602544952795E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:40">
+    <row r="56" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>27</v>
       </c>
@@ -5572,7 +5570,7 @@
         <v>1.5841957667984317E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:40">
+    <row r="57" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>50</v>
       </c>
@@ -5612,7 +5610,7 @@
         <v>1.7778128206867212E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:40">
+    <row r="58" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>29</v>
       </c>
@@ -5673,7 +5671,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N51"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.28515625" customWidth="1"/>
     <col min="2" max="13" width="10.42578125" customWidth="1"/>
@@ -5697,12 +5695,12 @@
     <col min="36" max="37" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>0</v>
       </c>
@@ -5746,7 +5744,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -5790,7 +5788,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -5822,7 +5820,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -5866,7 +5864,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -5898,7 +5896,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -5943,7 +5941,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>39</v>
       </c>
@@ -5975,7 +5973,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -6019,7 +6017,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -6051,63 +6049,63 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="39">
-        <f>(stock!$W$36*'Rel. eff.'!B12+stock!$W$50*'Rel. eff.'!B14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!B12+stock!$W$50*'Rel. eff.'!B16)/stock!$W$18</f>
         <v>3.5787823946793083</v>
       </c>
       <c r="C11" s="39">
-        <f>(stock!$W$36*'Rel. eff.'!C12+stock!$W$50*'Rel. eff.'!C14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!C12+stock!$W$50*'Rel. eff.'!C16)/stock!$W$18</f>
         <v>3.5787823946793083</v>
       </c>
       <c r="D11" s="39">
-        <f>(stock!$W$36*'Rel. eff.'!D12+stock!$W$50*'Rel. eff.'!D14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!D12+stock!$W$50*'Rel. eff.'!D16)/stock!$W$18</f>
         <v>3.5787823946793083</v>
       </c>
       <c r="E11" s="14">
-        <f>(stock!$W$36*'Rel. eff.'!E12+stock!$W$50*'Rel. eff.'!E14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!E12+stock!$W$50*'Rel. eff.'!E16)/stock!$W$18</f>
         <v>3.5787823946793083</v>
       </c>
       <c r="F11" s="14">
-        <f>(stock!$W$36*'Rel. eff.'!F12+stock!$W$50*'Rel. eff.'!F14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!F12+stock!$W$50*'Rel. eff.'!F16)/stock!$W$18</f>
         <v>3.718235194419762</v>
       </c>
       <c r="G11" s="14">
-        <f>(stock!$W$36*'Rel. eff.'!G12+stock!$W$50*'Rel. eff.'!G14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!G12+stock!$W$50*'Rel. eff.'!G16)/stock!$W$18</f>
         <v>3.718235194419762</v>
       </c>
       <c r="H11" s="33">
-        <f>(stock!$W$36*'Rel. eff.'!H12+stock!$W$50*'Rel. eff.'!H14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!H12+stock!$W$50*'Rel. eff.'!H16)/stock!$W$18</f>
         <v>3.718235194419762</v>
       </c>
       <c r="I11" s="32">
-        <f>(stock!$W$36*'Rel. eff.'!I12+stock!$W$50*'Rel. eff.'!I14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!I12+stock!$W$50*'Rel. eff.'!I16)/stock!$W$18</f>
         <v>3.718235194419762</v>
       </c>
       <c r="J11" s="32">
-        <f>(stock!$W$36*'Rel. eff.'!J12+stock!$W$50*'Rel. eff.'!J14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!J12+stock!$W$50*'Rel. eff.'!J16)/stock!$W$18</f>
         <v>3.718235194419762</v>
       </c>
       <c r="K11" s="32">
-        <f>(stock!$W$36*'Rel. eff.'!K12+stock!$W$50*'Rel. eff.'!K14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!K12+stock!$W$50*'Rel. eff.'!K16)/stock!$W$18</f>
         <v>3.718235194419762</v>
       </c>
       <c r="L11" s="32">
-        <f>(stock!$W$36*'Rel. eff.'!L12+stock!$W$50*'Rel. eff.'!L14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!L12+stock!$W$50*'Rel. eff.'!L16)/stock!$W$18</f>
         <v>3.718235194419762</v>
       </c>
       <c r="M11" s="32">
-        <f>(stock!$W$36*'Rel. eff.'!M12+stock!$W$50*'Rel. eff.'!M14)/stock!$W$18</f>
+        <f>(stock!$W$36*'Rel. eff.'!M12+stock!$W$50*'Rel. eff.'!M16)/stock!$W$18</f>
         <v>3.718235194419762</v>
       </c>
       <c r="N11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -6151,7 +6149,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -6183,7 +6181,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -6227,7 +6225,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>44</v>
       </c>
@@ -6259,7 +6257,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -6303,7 +6301,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>45</v>
       </c>
@@ -6335,63 +6333,63 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>46</v>
       </c>
       <c r="B18" s="44">
-        <f>(stock!$W$37*'Rel. eff.'!B19+0.293071*stock!$W$51*'Rel. eff.'!B21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!B19+0.293071*stock!$W$51*'Rel. eff.'!B23)/stock!$W$19</f>
         <v>566.54833238201707</v>
       </c>
       <c r="C18" s="44">
-        <f>(stock!$W$37*'Rel. eff.'!C19+0.293071*stock!$W$51*'Rel. eff.'!C21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!C19+0.293071*stock!$W$51*'Rel. eff.'!C23)/stock!$W$19</f>
         <v>566.54833238201707</v>
       </c>
       <c r="D18" s="44">
-        <f>(stock!$W$37*'Rel. eff.'!D19+0.293071*stock!$W$51*'Rel. eff.'!D21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!D19+0.293071*stock!$W$51*'Rel. eff.'!D23)/stock!$W$19</f>
         <v>566.54833238201707</v>
       </c>
-      <c r="E18" s="12">
-        <f>(stock!$W$37*'Rel. eff.'!E19+0.293071*stock!$W$51*'Rel. eff.'!E21)/stock!$W$19</f>
+      <c r="E18" s="44">
+        <f>(stock!$W$37*'Rel. eff.'!E19+0.293071*stock!$W$51*'Rel. eff.'!E23)/stock!$W$19</f>
         <v>566.54833238201707</v>
       </c>
-      <c r="F18" s="12">
-        <f>(stock!$W$37*'Rel. eff.'!F19+0.293071*stock!$W$51*'Rel. eff.'!F21)/stock!$W$19</f>
+      <c r="F18" s="44">
+        <f>(stock!$W$37*'Rel. eff.'!F19+0.293071*stock!$W$51*'Rel. eff.'!F23)/stock!$W$19</f>
         <v>557.18471341355928</v>
       </c>
       <c r="G18" s="12">
-        <f>(stock!$W$37*'Rel. eff.'!G19+0.293071*stock!$W$51*'Rel. eff.'!G21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!G19+0.293071*stock!$W$51*'Rel. eff.'!G23)/stock!$W$19</f>
         <v>557.18471341355928</v>
       </c>
       <c r="H18" s="37">
-        <f>(stock!$W$37*'Rel. eff.'!H19+0.293071*stock!$W$51*'Rel. eff.'!H21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!H19+0.293071*stock!$W$51*'Rel. eff.'!H23)/stock!$W$19</f>
         <v>557.18471341355928</v>
       </c>
       <c r="I18" s="38">
-        <f>(stock!$W$37*'Rel. eff.'!I19+0.293071*stock!$W$51*'Rel. eff.'!I21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!I19+0.293071*stock!$W$51*'Rel. eff.'!I23)/stock!$W$19</f>
         <v>557.18471341355928</v>
       </c>
       <c r="J18" s="38">
-        <f>(stock!$W$37*'Rel. eff.'!J19+0.293071*stock!$W$51*'Rel. eff.'!J21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!J19+0.293071*stock!$W$51*'Rel. eff.'!J23)/stock!$W$19</f>
         <v>557.18471341355928</v>
       </c>
       <c r="K18" s="38">
-        <f>(stock!$W$37*'Rel. eff.'!K19+0.293071*stock!$W$51*'Rel. eff.'!K21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!K19+0.293071*stock!$W$51*'Rel. eff.'!K23)/stock!$W$19</f>
         <v>557.18471341355928</v>
       </c>
       <c r="L18" s="38">
-        <f>(stock!$W$37*'Rel. eff.'!L19+0.293071*stock!$W$51*'Rel. eff.'!L21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!L19+0.293071*stock!$W$51*'Rel. eff.'!L23)/stock!$W$19</f>
         <v>557.18471341355928</v>
       </c>
       <c r="M18" s="38">
-        <f>(stock!$W$37*'Rel. eff.'!M19+0.293071*stock!$W$51*'Rel. eff.'!M21)/stock!$W$19</f>
+        <f>(stock!$W$37*'Rel. eff.'!M19+0.293071*stock!$W$51*'Rel. eff.'!M23)/stock!$W$19</f>
         <v>557.18471341355928</v>
       </c>
       <c r="N18" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -6435,7 +6433,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>47</v>
       </c>
@@ -6467,7 +6465,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -6511,7 +6509,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>49</v>
       </c>
@@ -6543,7 +6541,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -6587,7 +6585,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>50</v>
       </c>
@@ -6619,7 +6617,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -6634,12 +6632,12 @@
       <c r="L25" s="38"/>
       <c r="M25" s="38"/>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="27" t="s">
         <v>0</v>
       </c>
@@ -6683,7 +6681,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -6739,7 +6737,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -6777,7 +6775,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>17</v>
       </c>
@@ -6833,7 +6831,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>38</v>
       </c>
@@ -6871,7 +6869,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>18</v>
       </c>
@@ -6927,7 +6925,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>39</v>
       </c>
@@ -6965,7 +6963,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>19</v>
       </c>
@@ -7021,7 +7019,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -7059,7 +7057,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -7115,7 +7113,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>21</v>
       </c>
@@ -7171,7 +7169,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>42</v>
       </c>
@@ -7209,7 +7207,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>43</v>
       </c>
@@ -7265,7 +7263,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>44</v>
       </c>
@@ -7303,7 +7301,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>23</v>
       </c>
@@ -7359,7 +7357,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>45</v>
       </c>
@@ -7397,7 +7395,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>46</v>
       </c>
@@ -7453,7 +7451,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>25</v>
       </c>
@@ -7509,7 +7507,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>47</v>
       </c>
@@ -7547,7 +7545,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>48</v>
       </c>
@@ -7603,7 +7601,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>49</v>
       </c>
@@ -7641,7 +7639,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>27</v>
       </c>
@@ -7697,7 +7695,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>50</v>
       </c>
@@ -7735,7 +7733,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>29</v>
       </c>
@@ -7781,13 +7779,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:W57"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="54" style="1" customWidth="1"/>
@@ -7798,11 +7797,11 @@
     <col min="23" max="23" width="9.140625" style="25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="45.2" customHeight="1"/>
-    <row r="2" spans="1:23" ht="34.5" customHeight="1">
+    <row r="1" spans="1:23" ht="45.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:23" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2"/>
     </row>
-    <row r="5" spans="1:23" ht="13.5" customHeight="1">
+    <row r="5" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>61</v>
       </c>
@@ -7817,7 +7816,7 @@
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
     </row>
-    <row r="6" spans="1:23" ht="13.5" customHeight="1">
+    <row r="6" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -7830,7 +7829,7 @@
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
     </row>
-    <row r="7" spans="1:23" ht="16.5" customHeight="1">
+    <row r="7" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>62</v>
       </c>
@@ -7838,19 +7837,19 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:23" s="5" customFormat="1" ht="13.5" customHeight="1">
+    <row r="8" spans="1:23" s="5" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B8" s="1"/>
       <c r="W8" s="4"/>
     </row>
-    <row r="9" spans="1:23" ht="13.5" customHeight="1">
+    <row r="9" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
     </row>
-    <row r="10" spans="1:23" ht="13.5" customHeight="1"/>
-    <row r="11" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
+    <row r="10" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:23" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="7">
         <v>2000</v>
       </c>
@@ -7915,13 +7914,13 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="13.5" customHeight="1"/>
-    <row r="13" spans="1:23" ht="13.5" customHeight="1">
+    <row r="12" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="13.5" customHeight="1">
+    <row r="14" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>2</v>
       </c>
@@ -7989,7 +7988,7 @@
         <v>7185.5439999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="13.5" customHeight="1">
+    <row r="15" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
         <v>3</v>
       </c>
@@ -8057,7 +8056,7 @@
         <v>2820.4940000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="13.5" customHeight="1">
+    <row r="16" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
         <v>4</v>
       </c>
@@ -8125,7 +8124,7 @@
         <v>3212.2289999999998</v>
       </c>
     </row>
-    <row r="17" spans="2:23" ht="13.5" customHeight="1">
+    <row r="17" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
         <v>5</v>
       </c>
@@ -8193,7 +8192,7 @@
         <v>4247.5290000000005</v>
       </c>
     </row>
-    <row r="18" spans="2:23" ht="13.5" customHeight="1">
+    <row r="18" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
         <v>6</v>
       </c>
@@ -8261,7 +8260,7 @@
         <v>4401.5330000000004</v>
       </c>
     </row>
-    <row r="19" spans="2:23" ht="13.5" customHeight="1">
+    <row r="19" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="9" t="s">
         <v>7</v>
       </c>
@@ -8329,7 +8328,7 @@
         <v>5596.2179999999998</v>
       </c>
     </row>
-    <row r="20" spans="2:23" ht="13.5" customHeight="1">
+    <row r="20" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
         <v>28</v>
       </c>
@@ -8397,7 +8396,7 @@
         <v>108146.92200000001</v>
       </c>
     </row>
-    <row r="21" spans="2:23" ht="13.5" customHeight="1">
+    <row r="21" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="11"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
@@ -8421,12 +8420,12 @@
       <c r="V21" s="12"/>
       <c r="W21" s="38"/>
     </row>
-    <row r="22" spans="2:23" ht="13.5" customHeight="1">
+    <row r="22" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="8" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="2:23" ht="13.5" customHeight="1">
+    <row r="23" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="13" t="s">
         <v>2</v>
       </c>
@@ -8494,7 +8493,7 @@
         <v>1.284</v>
       </c>
     </row>
-    <row r="24" spans="2:23" ht="13.5" customHeight="1">
+    <row r="24" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="13" t="s">
         <v>3</v>
       </c>
@@ -8562,7 +8561,7 @@
         <v>0.504</v>
       </c>
     </row>
-    <row r="25" spans="2:23" ht="13.5" customHeight="1">
+    <row r="25" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="13" t="s">
         <v>4</v>
       </c>
@@ -8630,7 +8629,7 @@
         <v>0.57399999999999995</v>
       </c>
     </row>
-    <row r="26" spans="2:23" ht="13.5" customHeight="1">
+    <row r="26" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="13" t="s">
         <v>5</v>
       </c>
@@ -8698,7 +8697,7 @@
         <v>0.75900000000000001</v>
       </c>
     </row>
-    <row r="27" spans="2:23" ht="13.5" customHeight="1">
+    <row r="27" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="13" t="s">
         <v>6</v>
       </c>
@@ -8766,7 +8765,7 @@
         <v>0.78651899999999997</v>
       </c>
     </row>
-    <row r="28" spans="2:23" ht="13.5" customHeight="1">
+    <row r="28" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="13" t="s">
         <v>7</v>
       </c>
@@ -8834,7 +8833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:23" ht="13.5" customHeight="1">
+    <row r="29" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="9" t="s">
         <v>28</v>
       </c>
@@ -8902,15 +8901,15 @@
         <v>19.324999999999999</v>
       </c>
     </row>
-    <row r="30" spans="2:23" ht="13.5" customHeight="1">
+    <row r="30" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="11"/>
     </row>
-    <row r="31" spans="2:23" ht="13.5" customHeight="1">
+    <row r="31" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="15" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="32" spans="2:23" ht="13.5" customHeight="1">
+    <row r="32" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="13" t="s">
         <v>2</v>
       </c>
@@ -8978,7 +8977,7 @@
         <v>7185.5439999999999</v>
       </c>
     </row>
-    <row r="33" spans="2:23" ht="13.5" customHeight="1">
+    <row r="33" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="13" t="s">
         <v>3</v>
       </c>
@@ -9046,7 +9045,7 @@
         <v>2820.4940000000001</v>
       </c>
     </row>
-    <row r="34" spans="2:23" ht="13.5" customHeight="1">
+    <row r="34" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="13" t="s">
         <v>4</v>
       </c>
@@ -9114,7 +9113,7 @@
         <v>3212.2289999999998</v>
       </c>
     </row>
-    <row r="35" spans="2:23" ht="13.5" customHeight="1">
+    <row r="35" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="13" t="s">
         <v>5</v>
       </c>
@@ -9182,7 +9181,7 @@
         <v>4247.5290000000005</v>
       </c>
     </row>
-    <row r="36" spans="2:23" ht="13.5" customHeight="1">
+    <row r="36" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="13" t="s">
         <v>6</v>
       </c>
@@ -9250,7 +9249,7 @@
         <v>4281.107</v>
       </c>
     </row>
-    <row r="37" spans="2:23" ht="13.5" customHeight="1">
+    <row r="37" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="13" t="s">
         <v>7</v>
       </c>
@@ -9318,7 +9317,7 @@
         <v>4801.5559999999996</v>
       </c>
     </row>
-    <row r="38" spans="2:23" ht="13.5" customHeight="1">
+    <row r="38" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="9" t="s">
         <v>28</v>
       </c>
@@ -9386,15 +9385,15 @@
         <v>108146.92200000001</v>
       </c>
     </row>
-    <row r="39" spans="2:23" ht="13.5" customHeight="1">
+    <row r="39" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="11"/>
     </row>
-    <row r="40" spans="2:23" ht="13.5" customHeight="1">
+    <row r="40" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="8" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="41" spans="2:23" ht="13.5" customHeight="1">
+    <row r="41" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="13" t="s">
         <v>2</v>
       </c>
@@ -9462,7 +9461,7 @@
         <v>1.284</v>
       </c>
     </row>
-    <row r="42" spans="2:23" ht="13.5" customHeight="1">
+    <row r="42" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="13" t="s">
         <v>3</v>
       </c>
@@ -9530,7 +9529,7 @@
         <v>0.504</v>
       </c>
     </row>
-    <row r="43" spans="2:23" ht="13.5" customHeight="1">
+    <row r="43" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="13" t="s">
         <v>4</v>
       </c>
@@ -9598,7 +9597,7 @@
         <v>0.57399999999999995</v>
       </c>
     </row>
-    <row r="44" spans="2:23" ht="13.5" customHeight="1">
+    <row r="44" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="13" t="s">
         <v>5</v>
       </c>
@@ -9666,7 +9665,7 @@
         <v>0.75900000000000001</v>
       </c>
     </row>
-    <row r="45" spans="2:23" ht="13.5" customHeight="1">
+    <row r="45" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="13" t="s">
         <v>6</v>
       </c>
@@ -9734,7 +9733,7 @@
         <v>0.76500000000000001</v>
       </c>
     </row>
-    <row r="46" spans="2:23" ht="13.5" customHeight="1">
+    <row r="46" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="13" t="s">
         <v>7</v>
       </c>
@@ -9802,7 +9801,7 @@
         <v>0.85799999999999998</v>
       </c>
     </row>
-    <row r="47" spans="2:23" ht="13.5" customHeight="1">
+    <row r="47" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="9" t="s">
         <v>28</v>
       </c>
@@ -9870,15 +9869,15 @@
         <v>19.324999999999999</v>
       </c>
     </row>
-    <row r="48" spans="2:23" ht="13.5" customHeight="1">
+    <row r="48" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="11"/>
     </row>
-    <row r="49" spans="1:23" ht="13.5" customHeight="1">
+    <row r="49" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="15" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="50" spans="1:23" ht="13.5" customHeight="1">
+    <row r="50" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="13" t="s">
         <v>6</v>
       </c>
@@ -9946,7 +9945,7 @@
         <v>120.426</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="13.5" customHeight="1">
+    <row r="51" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="13" t="s">
         <v>7</v>
       </c>
@@ -10014,15 +10013,15 @@
         <v>794.66300000000001</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="13.5" customHeight="1">
+    <row r="52" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="11"/>
     </row>
-    <row r="53" spans="1:23" ht="13.5" customHeight="1">
+    <row r="53" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="8" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="13.5" customHeight="1">
+    <row r="54" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="13" t="s">
         <v>6</v>
       </c>
@@ -10090,7 +10089,7 @@
         <v>2.1519E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="13.5" customHeight="1">
+    <row r="55" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="13" t="s">
         <v>7</v>
       </c>
@@ -10158,8 +10157,8 @@
         <v>0.14199999999999999</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="13.5" customHeight="1"/>
-    <row r="57" spans="1:23" ht="13.5" customHeight="1">
+    <row r="56" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="17" t="s">
         <v>70</v>
       </c>
@@ -10174,7 +10173,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:W69"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="47.7109375" style="1" customWidth="1"/>
@@ -10187,11 +10186,11 @@
     <col min="23" max="23" width="10.85546875" style="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="45.2" customHeight="1"/>
-    <row r="2" spans="1:23" ht="34.5" customHeight="1">
+    <row r="1" spans="1:23" ht="45.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:23" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2"/>
     </row>
-    <row r="5" spans="1:23" ht="13.5" customHeight="1">
+    <row r="5" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>61</v>
       </c>
@@ -10206,7 +10205,7 @@
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
     </row>
-    <row r="6" spans="1:23" ht="13.5" customHeight="1">
+    <row r="6" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -10219,7 +10218,7 @@
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
     </row>
-    <row r="7" spans="1:23" ht="16.5" customHeight="1">
+    <row r="7" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>71</v>
       </c>
@@ -10227,19 +10226,19 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:23" s="5" customFormat="1" ht="13.5" customHeight="1">
+    <row r="8" spans="1:23" s="5" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>72</v>
       </c>
       <c r="B8" s="1"/>
       <c r="W8" s="4"/>
     </row>
-    <row r="9" spans="1:23" ht="13.5" customHeight="1">
+    <row r="9" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
     </row>
-    <row r="10" spans="1:23" ht="13.5" customHeight="1"/>
-    <row r="11" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
+    <row r="10" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:23" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="7">
         <v>2000</v>
       </c>
@@ -10304,8 +10303,8 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="13.5" customHeight="1"/>
-    <row r="13" spans="1:23" s="18" customFormat="1" ht="13.5" customHeight="1">
+    <row r="12" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:23" s="18" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="15" t="s">
         <v>73</v>
       </c>
@@ -10373,7 +10372,7 @@
         <v>63.938434000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="13.5" customHeight="1">
+    <row r="14" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="20" t="s">
         <v>74</v>
       </c>
@@ -10399,7 +10398,7 @@
       <c r="V14" s="16"/>
       <c r="W14" s="36"/>
     </row>
-    <row r="15" spans="1:23" ht="13.5" customHeight="1">
+    <row r="15" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="13" t="s">
         <v>2</v>
       </c>
@@ -10467,7 +10466,7 @@
         <v>8.6857009999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="13.5" customHeight="1">
+    <row r="16" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="13" t="s">
         <v>3</v>
       </c>
@@ -10535,7 +10534,7 @@
         <v>2.7517200000000002</v>
       </c>
     </row>
-    <row r="17" spans="2:23" ht="13.5" customHeight="1">
+    <row r="17" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="13" t="s">
         <v>75</v>
       </c>
@@ -10603,7 +10602,7 @@
         <v>0.65966899999999995</v>
       </c>
     </row>
-    <row r="18" spans="2:23" ht="13.5" customHeight="1">
+    <row r="18" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="13" t="s">
         <v>76</v>
       </c>
@@ -10671,7 +10670,7 @@
         <v>0.42840899999999998</v>
       </c>
     </row>
-    <row r="19" spans="2:23" ht="13.5" customHeight="1">
+    <row r="19" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="13" t="s">
         <v>6</v>
       </c>
@@ -10739,7 +10738,7 @@
         <v>10.28895</v>
       </c>
     </row>
-    <row r="20" spans="2:23" ht="13.5" customHeight="1">
+    <row r="20" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="13" t="s">
         <v>7</v>
       </c>
@@ -10807,7 +10806,7 @@
         <v>10.940383000000001</v>
       </c>
     </row>
-    <row r="21" spans="2:23" ht="13.5" customHeight="1">
+    <row r="21" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="9" t="s">
         <v>77</v>
       </c>
@@ -10875,7 +10874,7 @@
         <v>30.183602</v>
       </c>
     </row>
-    <row r="22" spans="2:23" ht="13.5" customHeight="1">
+    <row r="22" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="11"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
@@ -10899,7 +10898,7 @@
       <c r="V22" s="16"/>
       <c r="W22" s="36"/>
     </row>
-    <row r="23" spans="2:23" ht="13.5" customHeight="1">
+    <row r="23" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="20" t="s">
         <v>78</v>
       </c>
@@ -10925,7 +10924,7 @@
       <c r="V23" s="16"/>
       <c r="W23" s="36"/>
     </row>
-    <row r="24" spans="2:23" ht="13.5" customHeight="1">
+    <row r="24" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="13" t="s">
         <v>2</v>
       </c>
@@ -10993,7 +10992,7 @@
         <v>13.584476</v>
       </c>
     </row>
-    <row r="25" spans="2:23" ht="13.5" customHeight="1">
+    <row r="25" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="13" t="s">
         <v>3</v>
       </c>
@@ -11061,7 +11060,7 @@
         <v>4.3037029999999996</v>
       </c>
     </row>
-    <row r="26" spans="2:23" ht="13.5" customHeight="1">
+    <row r="26" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="13" t="s">
         <v>75</v>
       </c>
@@ -11129,7 +11128,7 @@
         <v>1.0317259999999999</v>
       </c>
     </row>
-    <row r="27" spans="2:23" ht="13.5" customHeight="1">
+    <row r="27" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="13" t="s">
         <v>76</v>
       </c>
@@ -11197,7 +11196,7 @@
         <v>0.67003400000000002</v>
       </c>
     </row>
-    <row r="28" spans="2:23" ht="13.5" customHeight="1">
+    <row r="28" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="13" t="s">
         <v>6</v>
       </c>
@@ -11265,7 +11264,7 @@
         <v>16.091963</v>
       </c>
     </row>
-    <row r="29" spans="2:23" ht="13.5" customHeight="1">
+    <row r="29" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="13" t="s">
         <v>7</v>
       </c>
@@ -11333,7 +11332,7 @@
         <v>17.110809</v>
       </c>
     </row>
-    <row r="30" spans="2:23" ht="13.5" customHeight="1">
+    <row r="30" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="9" t="s">
         <v>77</v>
       </c>
@@ -11401,15 +11400,15 @@
         <v>47.207290999999998</v>
       </c>
     </row>
-    <row r="31" spans="2:23" ht="13.5" customHeight="1">
+    <row r="31" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="11"/>
     </row>
-    <row r="32" spans="2:23" ht="13.5" customHeight="1">
+    <row r="32" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="21" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="33" spans="2:23" ht="13.5" customHeight="1">
+    <row r="33" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="22" t="s">
         <v>80</v>
       </c>
@@ -11477,10 +11476,10 @@
         <v>5596.2179999999998</v>
       </c>
     </row>
-    <row r="34" spans="2:23" ht="13.5" customHeight="1">
+    <row r="34" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="11"/>
     </row>
-    <row r="35" spans="2:23" s="18" customFormat="1" ht="13.5" customHeight="1">
+    <row r="35" spans="2:23" s="18" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="21" t="s">
         <v>81</v>
       </c>
@@ -11548,7 +11547,7 @@
         <v>11.425293</v>
       </c>
     </row>
-    <row r="36" spans="2:23" ht="13.5" customHeight="1">
+    <row r="36" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="11"/>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
@@ -11572,7 +11571,7 @@
       <c r="V36" s="16"/>
       <c r="W36" s="36"/>
     </row>
-    <row r="37" spans="2:23" ht="13.5" customHeight="1">
+    <row r="37" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="11"/>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
@@ -11596,7 +11595,7 @@
       <c r="V37" s="16"/>
       <c r="W37" s="36"/>
     </row>
-    <row r="38" spans="2:23" s="18" customFormat="1" ht="30" customHeight="1">
+    <row r="38" spans="2:23" s="18" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="8" t="s">
         <v>82</v>
       </c>
@@ -11664,7 +11663,7 @@
         <v>0.20105500000000001</v>
       </c>
     </row>
-    <row r="39" spans="2:23" ht="13.5" customHeight="1">
+    <row r="39" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="20" t="s">
         <v>83</v>
       </c>
@@ -11690,7 +11689,7 @@
       <c r="V39" s="16"/>
       <c r="W39" s="36"/>
     </row>
-    <row r="40" spans="2:23" ht="13.5" customHeight="1">
+    <row r="40" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="13" t="s">
         <v>2</v>
       </c>
@@ -11758,7 +11757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:23" ht="13.5" customHeight="1">
+    <row r="41" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="13" t="s">
         <v>3</v>
       </c>
@@ -11826,7 +11825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:23" ht="13.5" customHeight="1">
+    <row r="42" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="13" t="s">
         <v>75</v>
       </c>
@@ -11894,7 +11893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:23" ht="13.5" customHeight="1">
+    <row r="43" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="13" t="s">
         <v>76</v>
       </c>
@@ -11962,7 +11961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:23" ht="13.5" customHeight="1">
+    <row r="44" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="13" t="s">
         <v>6</v>
       </c>
@@ -12030,7 +12029,7 @@
         <v>1.9727999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="2:23" ht="13.5" customHeight="1">
+    <row r="45" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="13" t="s">
         <v>7</v>
       </c>
@@ -12098,7 +12097,7 @@
         <v>0.18132599999999999</v>
       </c>
     </row>
-    <row r="46" spans="2:23" ht="13.5" customHeight="1">
+    <row r="46" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="9" t="s">
         <v>77</v>
       </c>
@@ -12166,7 +12165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="2:23" ht="13.5" customHeight="1">
+    <row r="47" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="11"/>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
@@ -12190,7 +12189,7 @@
       <c r="V47" s="16"/>
       <c r="W47" s="36"/>
     </row>
-    <row r="48" spans="2:23" s="18" customFormat="1" ht="13.5" customHeight="1">
+    <row r="48" spans="2:23" s="18" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="15" t="s">
         <v>84</v>
       </c>
@@ -12258,7 +12257,7 @@
         <v>3.1445020000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:23" s="18" customFormat="1" ht="13.5" customHeight="1">
+    <row r="49" spans="1:23" s="18" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="15"/>
       <c r="C49" s="19"/>
       <c r="D49" s="19"/>
@@ -12282,7 +12281,7 @@
       <c r="V49" s="19"/>
       <c r="W49" s="19"/>
     </row>
-    <row r="50" spans="1:23" ht="13.5" customHeight="1">
+    <row r="50" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="11"/>
       <c r="C50" s="16"/>
       <c r="D50" s="16"/>
@@ -12306,7 +12305,7 @@
       <c r="V50" s="16"/>
       <c r="W50" s="36"/>
     </row>
-    <row r="51" spans="1:23" ht="13.5" customHeight="1">
+    <row r="51" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="15" t="s">
         <v>85</v>
       </c>
@@ -12332,7 +12331,7 @@
       <c r="V51" s="16"/>
       <c r="W51" s="36"/>
     </row>
-    <row r="52" spans="1:23" ht="13.5" customHeight="1">
+    <row r="52" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="13" t="s">
         <v>2</v>
       </c>
@@ -12400,7 +12399,7 @@
         <v>3.1887439999999998</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="13.5" customHeight="1">
+    <row r="53" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="13" t="s">
         <v>3</v>
       </c>
@@ -12468,7 +12467,7 @@
         <v>1.010227</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="13.5" customHeight="1">
+    <row r="54" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="13" t="s">
         <v>75</v>
       </c>
@@ -12536,7 +12535,7 @@
         <v>8.0726999999999993E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="13.5" customHeight="1">
+    <row r="55" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="13" t="s">
         <v>76</v>
       </c>
@@ -12604,7 +12603,7 @@
         <v>8.7377999999999997E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="13.5" customHeight="1">
+    <row r="56" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="13" t="s">
         <v>6</v>
       </c>
@@ -12672,7 +12671,7 @@
         <v>1.049261</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="13.5" customHeight="1">
+    <row r="57" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="13" t="s">
         <v>7</v>
       </c>
@@ -12740,7 +12739,7 @@
         <v>3.3470800000000001</v>
       </c>
     </row>
-    <row r="58" spans="1:23">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B58" s="9" t="s">
         <v>86</v>
       </c>
@@ -12808,25 +12807,25 @@
         <v>11.081178</v>
       </c>
     </row>
-    <row r="60" spans="1:23">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B60"/>
     </row>
-    <row r="61" spans="1:23">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>88</v>
       </c>
       <c r="B61"/>
     </row>
-    <row r="62" spans="1:23">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B62"/>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" s="15"/>
     </row>
   </sheetData>

</xml_diff>